<commit_message>
Reworked project organization to leave sensitive materials on secure OneDrive server and export output to shared OneDrive folder
</commit_message>
<xml_diff>
--- a/docs/NOrmal ranges and Adverse Events grading system.xlsx
+++ b/docs/NOrmal ranges and Adverse Events grading system.xlsx
@@ -1783,8 +1783,8 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000C8DD2C9503A9346957BF8010701C0C0" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8fb9d6bcbce96ea4820cba4545c13952">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="44ad9495-3741-4708-b440-876241155999" xmlns:ns3="98305de1-6b4d-4e48-ba1d-6a2d8f079fc7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c86def3c84f9d4c2cb9156fbe4c263eb" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000C8DD2C9503A9346957BF8010701C0C0" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="36c570434a73bd4724d1e0329b0da23d">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="44ad9495-3741-4708-b440-876241155999" xmlns:ns3="98305de1-6b4d-4e48-ba1d-6a2d8f079fc7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="15d4c143b1ef6d1abf62619997e119eb" ns2:_="" ns3:_="">
     <xsd:import namespace="44ad9495-3741-4708-b440-876241155999"/>
     <xsd:import namespace="98305de1-6b4d-4e48-ba1d-6a2d8f079fc7"/>
     <xsd:element name="properties">
@@ -2037,7 +2037,7 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D70D4D42-AD63-4E8D-8AED-A464E220E0DC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F64D4BF1-4448-42F1-89FF-B5C97328C911}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>